<commit_message>
TEMP: drop resolve from one server line, to prove the guard fails CI
</commit_message>
<xml_diff>
--- a/planning/Master Plan API Gateway.xlsx
+++ b/planning/Master Plan API Gateway.xlsx
@@ -1233,16 +1233,17 @@
       </c>
       <c r="J7" s="55" t="inlineStr">
         <is>
-          <t>Đang làm. Môi trường ĐO đã dựng: LiteLLM 1.99.0 (fork litellm_rang_dong, commit f005afa146) trên Docker, 1 tuyến Google AI Studio. 31/08/2026 agent đầu tiên (DMS) đã chạy THẬT qua tuyến này: 45 lượt vào LiteLLM_SpendLogs (40 thành công / 5 hỏng). Còn 7 tuyến và 3 môi trường dev / staging / production.</t>
+          <t>Đang làm. Môi trường ĐO đã dựng: LiteLLM 1.99.0 (fork litellm_rang_dong, commit f005afa146) trên Docker, 1 tuyến Google AI Studio. 31/08/2026 agent đầu tiên (DMS) đã chạy THẬT qua tuyến này: 45 lượt vào LiteLLM_SpendLogs (40 thành công / 5 hỏng). Còn 7 tuyến và 3 môi trường dev / staging / production.
+15/09 GATEWAY THÔI BUILD TẠI CHỖ. Image đóng gói trong CI rồi đẩy lên kho GHCR (ghcr.io/ursweetheart/litellm_rang_dong), docker-compose.yml ghim đúng nhãn commit; CI báo đỏ nếu khối x-litellm còn build: hoặc ghim một nhãn không tồn tại. Bước build BẮT BUỘC có bản vá Sentinel trong fork, thiếu thì dừng. Trước đó đã ghi lại một lần build hỏng vì glibc lệch giữa máy build và máy chạy. 09/09 thêm tuyến thứ hai: Vertex express cho CRM (api_base kết thúc ở /publishers/google, không khai vertex_project — express tự suy). CÒN LẠI: 6 tuyến và 3 môi trường dev/staging/production. MỐC 14/09 ĐÃ TRÔI QUA MÀ CHƯA ĐẠT.</t>
         </is>
       </c>
       <c r="K7" s="17" t="n"/>
       <c r="L7" s="17" t="n"/>
       <c r="M7" s="17" t="n"/>
       <c r="N7" s="56" t="n"/>
-      <c r="O7" s="17" t="n"/>
-      <c r="P7" s="17" t="n"/>
-      <c r="Q7" s="17" t="n"/>
+      <c r="O7" s="56" t="n"/>
+      <c r="P7" s="56" t="n"/>
+      <c r="Q7" s="56" t="n"/>
       <c r="R7" s="17" t="n"/>
       <c r="S7" s="17" t="n"/>
       <c r="T7" s="17" t="n"/>
@@ -1292,7 +1293,8 @@
       </c>
       <c r="J8" s="55" t="inlineStr">
         <is>
-          <t>Xong 01/09/2026. 27/08 thêm vào docker-compose.yml (profile gateway): Redis 7 (1 primary + 1 replica), 2 instance LiteLLM stateless, nginx làm load balancer, database litellm riêng trên token-ledger-postgres. 31/08 nghiệm thu load balancer bằng lưu lượng thật của DMS. 01/09 nghiệm thu CACHE DÙNG CHUNG bằng một agent: hai request giống hệt nhau qua load balancer rơi vào HAI instance khác nhau, lượt hai trúng cache trên instance chưa từng ghi cache — 4.222 ms xuống 261 ms, cùng một id phản hồi, Redis giữ 13 khoá. Chứng minh trạng thái nằm ở Redis chứ không phải bộ nhớ từng tiến trình. Cache sau đó TẮT LẠI có chủ ý: đo được lượt trúng cache ghi spend = 0 nhưng VẪN ghi đủ 352 token, nên bật thật sẽ làm token qua Gateway phồng so với token Google tính tiền. Bật lại sau khi xong báo cáo đối chiếu bốn nguồn.</t>
+          <t>Xong 01/09/2026. 27/08 thêm vào docker-compose.yml (profile gateway): Redis 7 (1 primary + 1 replica), 2 instance LiteLLM stateless, nginx làm load balancer, database litellm riêng trên token-ledger-postgres. 31/08 nghiệm thu load balancer bằng lưu lượng thật của DMS. 01/09 nghiệm thu CACHE DÙNG CHUNG bằng một agent: hai request giống hệt nhau qua load balancer rơi vào HAI instance khác nhau, lượt hai trúng cache trên instance chưa từng ghi cache — 4.222 ms xuống 261 ms, cùng một id phản hồi, Redis giữ 13 khoá. Chứng minh trạng thái nằm ở Redis chứ không phải bộ nhớ từng tiến trình. Cache sau đó TẮT LẠI có chủ ý: đo được lượt trúng cache ghi spend = 0 nhưng VẪN ghi đủ 352 token, nên bật thật sẽ làm token qua Gateway phồng so với token Google tính tiền. Bật lại sau khi xong báo cáo đối chiếu bốn nguồn.
+08/09 THÊM SENTINEL — replica nay TỰ thăng cấp, không cần người. Nghiệm thu bằng cách GIẾT master thật, không phải xem tiến trình có lên không: 6 giây thì Sentinel trỏ sang địa chỉ mới, gọi thật ngay sau đó 10/10 lượt 200, p50 0,99 s p95 1,24 s — KHÔNG tệ hơn mốc trước khi giết (9/10 và p50 0,87 s). Chiều ngược (dựng lại master cũ) 7 giây, replica về làm slave. GHI RÕ ĐIỀU NÀY KHÔNG BẢO VỆ: ba sentinel nằm cùng MỘT máy, máy chết là chết tất — đây chưa phải tính sẵn sàng cao. Mức nghiêm trọng của vấn đề gốc là THẤP và đã đo 07/09 TRƯỚC khi quyết: tắt hẳn Redis thì Gateway vẫn phục vụ 9/10 lượt, p50 0,87 s, vì mọi thứ Redis giữ đều có TTL ≤ 60 giây.</t>
         </is>
       </c>
       <c r="K8" s="17" t="n"/>
@@ -1300,7 +1302,7 @@
       <c r="M8" s="17" t="n"/>
       <c r="N8" s="19" t="n"/>
       <c r="O8" s="19" t="n"/>
-      <c r="P8" s="17" t="n"/>
+      <c r="P8" s="53" t="n"/>
       <c r="Q8" s="17" t="n"/>
       <c r="R8" s="17" t="n"/>
       <c r="S8" s="17" t="n"/>
@@ -1361,15 +1363,16 @@
       </c>
       <c r="J9" s="55" t="inlineStr">
         <is>
-          <t>Đang làm. JWT đăng nhập đi qua Gateway nguyên vẹn (260 ký tự, đủ claim). 31/08 đã cấp Virtual Key ĐẦU TIÊN — cho DMS: 35/45 lượt mang khoá này. Đo được 9/45 lượt vẫn đi bằng master key (phép kiểm nội bộ) — loại này chỉ quy được về agent nhờ tag chứ không nhờ khoá, nên cần trường virtual_key_id để tách ra. Còn 7 khoá cho 7 agent và cơ chế thu hồi.</t>
+          <t>Đang làm. JWT đăng nhập đi qua Gateway nguyên vẹn (260 ký tự, đủ claim). 31/08 đã cấp Virtual Key ĐẦU TIÊN — cho DMS: 35/45 lượt mang khoá này. Đo được 9/45 lượt vẫn đi bằng master key (phép kiểm nội bộ) — loại này chỉ quy được về agent nhờ tag chứ không nhờ khoá, nên cần trường virtual_key_id để tách ra. Còn 7 khoá cho 7 agent và cơ chế thu hồi.
+07/09 API dashboard nay PHẢI có khoá mới đọc được. 09/09 đo trên khoá CRM: hai cửa chặn phân biệt được bằng mã — 403 là ngoài danh sách models của khoá, 401 là lọc tag. Danh sách models chạy TRƯỚC và ngắn mạch, nên một khoá đã hẹp thì phép kiểm lọc tag KHÔNG hề chạm tới; phải kiểm riêng bằng master key mới thấy lọc tag chạy đúng. Virtual Key: 2/8 (DMS, CRM). CÒN LẠI: 6 khoá và cơ chế thu hồi.</t>
         </is>
       </c>
       <c r="K9" s="17" t="n"/>
       <c r="L9" s="17" t="n"/>
       <c r="M9" s="17" t="n"/>
       <c r="N9" s="56" t="n"/>
-      <c r="O9" s="17" t="n"/>
-      <c r="P9" s="17" t="n"/>
+      <c r="O9" s="56" t="n"/>
+      <c r="P9" s="56" t="n"/>
       <c r="Q9" s="17" t="n"/>
       <c r="R9" s="17" t="n"/>
       <c r="S9" s="17" t="n"/>
@@ -1418,7 +1421,8 @@
       </c>
       <c r="J10" s="55" t="inlineStr">
         <is>
-          <t>Đo xong 26/08/2026: header khai ở user_header_name → cột end_user; toàn bộ header → proxy_server_request.metadata.headers (8/8 nguyên văn). Hiện trạng 01/09 trên 45 lượt: end_user mang 19 'svc.dms-feedback', 15 'tuan.tran' (phép thử đã rút lại), 11 rỗng — NHƯNG cả 41 dòng nạp được đều quy về đúng MỘT tài khoản 949 svc.dms-feedback, đúng quy ước 'agent một-người-dùng' chốt 20/08. CẦN CHỐT: quy ước định danh áp cho cả 8 agent hay chỉ cho 2 agent nhiều người dùng (TLA Hợp Đồng, Ralli).</t>
+          <t>Đo xong 26/08/2026: header khai ở user_header_name → cột end_user; toàn bộ header → proxy_server_request.metadata.headers (8/8 nguyên văn). Hiện trạng 01/09 trên 45 lượt: end_user mang 19 'svc.dms-feedback', 15 'tuan.tran' (phép thử đã rút lại), 11 rỗng — NHƯNG cả 41 dòng nạp được đều quy về đúng MỘT tài khoản 949 svc.dms-feedback, đúng quy ước 'agent một-người-dùng' chốt 20/08. CẦN CHỐT: quy ước định danh áp cho cả 8 agent hay chỉ cho 2 agent nhiều người dùng (TLA Hợp Đồng, Ralli).
+12/09 CRM lần ĐẦU có giá trị ở end_user: svc.crm-feedback (tài khoản 951) — trước nay usage_by_account có 0 dòng cho agent 7. Là định danh DỊCH VỤ, không bịa ra một con người. 13-15/09 soát danh tính trên 4 agent, chốt BA CHIỀU giữ riêng và không suy lẫn nhau: Virtual Key/tag xác định agent và tuyến được phép gọi; X-User xác định actor; phòng ban/đơn vị đến từ catalog — KHÔNG suy từ IP, tên khoá, hay dữ liệu client gửi lên. Mức xác minh KHÁC NHAU giữa các agent và không được cộng dồn: TLA-HĐ và Ralli đã xác minh CẢ X-User lẫn body user; DMS và CRM mới xác minh X-User → end_user.</t>
         </is>
       </c>
       <c r="K10" s="17" t="n"/>
@@ -1426,8 +1430,8 @@
       <c r="M10" s="17" t="n"/>
       <c r="N10" s="56" t="n"/>
       <c r="O10" s="17" t="n"/>
-      <c r="P10" s="17" t="n"/>
-      <c r="Q10" s="17" t="n"/>
+      <c r="P10" s="56" t="n"/>
+      <c r="Q10" s="56" t="n"/>
       <c r="R10" s="17" t="n"/>
       <c r="S10" s="17" t="n"/>
       <c r="T10" s="17" t="n"/>
@@ -1485,7 +1489,8 @@
       </c>
       <c r="J11" s="55" t="inlineStr">
         <is>
-          <t>Đang làm. 31/08 migration 006 thêm duration_ms, outcome, error_code — độ trễ 609–3.136 ms trên 38/38 lượt thành công; lượt hỏng ghi NULL vì LiteLLM ghi 0 cho MỌI lượt hỏng, kể cả lượt đã gọi tới Google. 01/09 migration 007 thêm nốt raw_model, virtual_key_id và cache_hit. ĐỐI CHIẾU 26 TRƯỜNG SHEET DATA OUT: 19/26 → 21/26, và 0 TRƯỜNG BẮT BUỘC CÒN THIẾU. Cả 12 trường mà mục này liệt kê đều đã có. 5 trường còn thiếu đều không bắt buộc (thinking_enabled, output_modality, cost_is_estimated, retry_count, fallback_used). Đo được khi nạp: 7/41 lượt (17,1%) đi bằng khoá quản trị chung chứ không phải khoá agent — trước khi có virtual_key_id thì không tách ra được. Nghiệm thu: 24/24 khoá mốc khớp, audit 42 phép kiểm / 38 đạt / 4 lưu ý / 0 hỏng. 03/09 migration 008 thêm output_modality và thinking_enabled — cả hai nằm CÙNG khối completion_tokens_details (bản đầu của đề xuất trỏ nhầm sang prompt_tokens_details; hai khối đều có text_tokens 42/42 nên đọc nhầm vẫn ra số, chỉ là số của chiều ngược lại). DATA OUT: 21/26 → 23/26 CÓ ĐƯỜNG NẠP — nhưng 2 trong 23 trường đó CHƯA CÓ SỐ, và cần đọc đúng như vậy: thinking_enabled 0/41 vì hai dòng duy nhất có reasoning_tokens (=342) không mang tag định danh agent nên bị loại ở khâu nạp (fact_call.agent_id là NOT NULL); cached_tokens 0/41, chưa kết luận được (đã loại trừ khả năng LiteLLM không ánh xạ; phép thử quyết định là hoá đơn ngày 31/08, chưa về). output_modality 38/41 — ba dòng rỗng là ba lượt hỏng, lượt hỏng không có phản hồi để dán nhãn. Bẫy đo được 03/09: DO UPDATE KHÔNG đủ khi thêm cột, phải chạy load_gateway.py --full, nếu không chỉ 6/41 dòng nhận cột mới. Nghiệm thu 03/09: 24/24 khoá mốc khớp, audit 54 phép kiểm / 50 đạt / 4 lưu ý / 0 hỏng. 05/09 ĐÍNH CHÍNH MỘT CÂU Ở TRÊN: dòng này viết "cached_tokens 0/41, chưa kết luận được ... phép thử quyết định là hoá đơn ngày 31/08". PHÉP THỬ ĐÓ KHÔNG THẮNG ĐƯỢC. Khoá của Gateway là FREE TIER — bằng chứng nằm ngay trong tên phép đo Google trả về (quota/generate_content_free_tier_input_token_count/usage, limit_name ...-FreeTier) — nên lưu lượng này sẽ KHÔNG BAO GIỜ lên hoá đơn, chờ bao lâu cũng vậy. Đường đối chiếu bắt buộc đi qua Cloud Monitoring, không qua fact_billing_daily. 05/09 ĐO ĐƯỢC MỘT KHOẢN THIẾU MÀ BẢN GHI KHÔNG NÓI RA: 12 trường mục này liệt kê đều CÓ MẶT, nhưng GIÁ TRỊ của chúng ở lượt hỏng là ĐIỀU SỔ KHAI chứ không phải ĐIỀU ĐÃ TIÊU. Ngày 31/08 nhà cung cấp báo 41 request với response_code = 200 cho TẤT CẢ, không một lỗi nào, trong khi sổ LiteLLM ghi 5 lượt hỏng — hai lượt đã được phục vụ xong và đã tiêu token thật, sổ ghi cho chúng 0 token 0 ms. Chênh 6.334 token = 12,29% của riêng ngày đó. Tên gọi: failed_is_not_free. load_gateway.py nay in token của lượt hỏng KÈM chữ "điều sổ khai", và audit_db.py nhóm I đối chiếu với số của nhà cung cấp. KHOẢN NỢ CÒN LẠI: 6 dòng sổ nguồn (760 token) không vào được fact_call, trong đó có một lượt THÀNH CÔNG 25 token, vì không có tag khớp dim_agent.code mà fact_call.agent_id là NOT NULL. Đã bác bỏ hai nghi can cũ (mốc nước, ranh giới ngày) bằng --full: vẫn inserted 0. Sửa được nó cần một agent "không quy được" hoặc agent_id cho phép NULL — chưa làm.</t>
+          <t>Đang làm. 31/08 migration 006 thêm duration_ms, outcome, error_code — độ trễ 609–3.136 ms trên 38/38 lượt thành công; lượt hỏng ghi NULL vì LiteLLM ghi 0 cho MỌI lượt hỏng, kể cả lượt đã gọi tới Google. 01/09 migration 007 thêm nốt raw_model, virtual_key_id và cache_hit. ĐỐI CHIẾU 26 TRƯỜNG SHEET DATA OUT: 19/26 → 21/26, và 0 TRƯỜNG BẮT BUỘC CÒN THIẾU. Cả 12 trường mà mục này liệt kê đều đã có. 5 trường còn thiếu đều không bắt buộc (thinking_enabled, output_modality, cost_is_estimated, retry_count, fallback_used). Đo được khi nạp: 7/41 lượt (17,1%) đi bằng khoá quản trị chung chứ không phải khoá agent — trước khi có virtual_key_id thì không tách ra được. Nghiệm thu: 24/24 khoá mốc khớp, audit 42 phép kiểm / 38 đạt / 4 lưu ý / 0 hỏng. 03/09 migration 008 thêm output_modality và thinking_enabled — cả hai nằm CÙNG khối completion_tokens_details (bản đầu của đề xuất trỏ nhầm sang prompt_tokens_details; hai khối đều có text_tokens 42/42 nên đọc nhầm vẫn ra số, chỉ là số của chiều ngược lại). DATA OUT: 21/26 → 23/26 CÓ ĐƯỜNG NẠP — nhưng 2 trong 23 trường đó CHƯA CÓ SỐ, và cần đọc đúng như vậy: thinking_enabled 0/41 vì hai dòng duy nhất có reasoning_tokens (=342) không mang tag định danh agent nên bị loại ở khâu nạp (fact_call.agent_id là NOT NULL); cached_tokens 0/41, chưa kết luận được (đã loại trừ khả năng LiteLLM không ánh xạ; phép thử quyết định là hoá đơn ngày 31/08, chưa về). output_modality 38/41 — ba dòng rỗng là ba lượt hỏng, lượt hỏng không có phản hồi để dán nhãn. Bẫy đo được 03/09: DO UPDATE KHÔNG đủ khi thêm cột, phải chạy load_gateway.py --full, nếu không chỉ 6/41 dòng nhận cột mới. Nghiệm thu 03/09: 24/24 khoá mốc khớp, audit 54 phép kiểm / 50 đạt / 4 lưu ý / 0 hỏng. 05/09 ĐÍNH CHÍNH MỘT CÂU Ở TRÊN: dòng này viết "cached_tokens 0/41, chưa kết luận được ... phép thử quyết định là hoá đơn ngày 31/08". PHÉP THỬ ĐÓ KHÔNG THẮNG ĐƯỢC. Khoá của Gateway là FREE TIER — bằng chứng nằm ngay trong tên phép đo Google trả về (quota/generate_content_free_tier_input_token_count/usage, limit_name ...-FreeTier) — nên lưu lượng này sẽ KHÔNG BAO GIỜ lên hoá đơn, chờ bao lâu cũng vậy. Đường đối chiếu bắt buộc đi qua Cloud Monitoring, không qua fact_billing_daily. 05/09 ĐO ĐƯỢC MỘT KHOẢN THIẾU MÀ BẢN GHI KHÔNG NÓI RA: 12 trường mục này liệt kê đều CÓ MẶT, nhưng GIÁ TRỊ của chúng ở lượt hỏng là ĐIỀU SỔ KHAI chứ không phải ĐIỀU ĐÃ TIÊU. Ngày 31/08 nhà cung cấp báo 41 request với response_code = 200 cho TẤT CẢ, không một lỗi nào, trong khi sổ LiteLLM ghi 5 lượt hỏng — hai lượt đã được phục vụ xong và đã tiêu token thật, sổ ghi cho chúng 0 token 0 ms. Chênh 6.334 token = 12,29% của riêng ngày đó. Tên gọi: failed_is_not_free. load_gateway.py nay in token của lượt hỏng KÈM chữ "điều sổ khai", và audit_db.py nhóm I đối chiếu với số của nhà cung cấp. KHOẢN NỢ CÒN LẠI: 6 dòng sổ nguồn (760 token) không vào được fact_call, trong đó có một lượt THÀNH CÔNG 25 token, vì không có tag khớp dim_agent.code mà fact_call.agent_id là NOT NULL. Đã bác bỏ hai nghi can cũ (mốc nước, ranh giới ngày) bằng --full: vẫn inserted 0. Sửa được nó cần một agent "không quy được" hoặc agent_id cho phép NULL — chưa làm.
+11/09 CHỐT TOKEN SUY NGHĨ: hoá đơn tính reasoning_tokens là token ĐẦU RA, không phải một loại thứ ba. Đường ống từng giả vờ ngược lại đã XOÁ, và cột được đặt tên theo đúng thứ nó đếm. 11/09 ĐO ranh giới ngày hoá đơn thay vì suy ra: ngày để nguyên giờ Pacific và ghim bằng một phép kiểm, sau khi đo được KHÔNG phép dịch múi giờ nào cho ra khớp toàn bộ — dịch cột ngày là chữa triệu chứng. 11/09 đọc nốt các cột Gateway còn bỏ qua. Nghiệm thu: 79 phép kiểm / 69 đạt / 10 lưu ý / 0 hỏng.</t>
         </is>
       </c>
       <c r="K11" s="17" t="n"/>
@@ -1493,7 +1498,7 @@
       <c r="M11" s="17" t="n"/>
       <c r="N11" s="56" t="n"/>
       <c r="O11" s="56" t="n"/>
-      <c r="P11" s="17" t="n"/>
+      <c r="P11" s="56" t="n"/>
       <c r="Q11" s="17" t="n"/>
       <c r="R11" s="17" t="n"/>
       <c r="S11" s="17" t="n"/>
@@ -1543,7 +1548,8 @@
       </c>
       <c r="J12" s="55" t="inlineStr">
         <is>
-          <t>Xong 03/09/2026, sớm 27 ngày so với mốc. Nhưng số thô đã sẵn sàng từ 31/08: fact_call.duration_ms giữ độ trễ TỪNG LƯỢT, nên p50/p95/p99 theo ngày tính lại được chính xác thay vì nội suy từ histogram gộp — thùng histogram của nguồn monitoring rộng 33,6 giây, mọi phân vị rút từ nó mang sai số hàng chục giây. Quy ước dữ liệu (ngày theo giờ VN, trường không đo được ghi NULL) đã áp dụng ở migration 006. Migration 008 dựng fact_usage_hourly — cùng năm chiều khoá như bảng ngày, chỉ đổi day thành hour: 3.327 dòng trên 1.751 giờ / 153 ngày (monitoring 2.624 · app 698 · gateway 5). KHÔNG có nguồn billing và đó là có chủ ý: hoá đơn Google chỉ tính theo NGÀY, chia đều cho 24 giờ sẽ cho ra một con số bịa — người đọc biết nguồn nào vắng bằng cách truy vấn cột source. Tổng theo giờ khớp tổng theo ngày cho TỪNG NGUỒN (bộ dựng tự dừng nếu lệch). Endpoint GET /api/usage-hourly, BẮT BUỘC có khoảng thời gian, khác 9 endpoint kia. Phân vị Gateway nay tính CHÍNH XÁC từ duration_ms thô: p95 ngày 31/08 = 1,822 s, khớp đúng con số change 006 tính tay; hai cột p95_bucket_* để NULL vì số thô không có sai số nội suy. Mỗi nguồn một dòng, không gộp trung bình. Chưa giải thích được: hai nguồn lệch 31,9 lần cho cùng agent 6 (thủ công p95 58,206 s vs gateway 1,822 s) và chưa ngày nào hai nguồn cùng có số để kiểm chứng lẫn nhau.</t>
+          <t>Xong 03/09/2026, sớm 27 ngày so với mốc. Nhưng số thô đã sẵn sàng từ 31/08: fact_call.duration_ms giữ độ trễ TỪNG LƯỢT, nên p50/p95/p99 theo ngày tính lại được chính xác thay vì nội suy từ histogram gộp — thùng histogram của nguồn monitoring rộng 33,6 giây, mọi phân vị rút từ nó mang sai số hàng chục giây. Quy ước dữ liệu (ngày theo giờ VN, trường không đo được ghi NULL) đã áp dụng ở migration 006. Migration 008 dựng fact_usage_hourly — cùng năm chiều khoá như bảng ngày, chỉ đổi day thành hour: 3.327 dòng trên 1.751 giờ / 153 ngày (monitoring 2.624 · app 698 · gateway 5). KHÔNG có nguồn billing và đó là có chủ ý: hoá đơn Google chỉ tính theo NGÀY, chia đều cho 24 giờ sẽ cho ra một con số bịa — người đọc biết nguồn nào vắng bằng cách truy vấn cột source. Tổng theo giờ khớp tổng theo ngày cho TỪNG NGUỒN (bộ dựng tự dừng nếu lệch). Endpoint GET /api/usage-hourly, BẮT BUỘC có khoảng thời gian, khác 9 endpoint kia. Phân vị Gateway nay tính CHÍNH XÁC từ duration_ms thô: p95 ngày 31/08 = 1,822 s, khớp đúng con số change 006 tính tay; hai cột p95_bucket_* để NULL vì số thô không có sai số nội suy. Mỗi nguồn một dòng, không gộp trung bình. Chưa giải thích được: hai nguồn lệch 31,9 lần cho cùng agent 6 (thủ công p95 58,206 s vs gateway 1,822 s) và chưa ngày nào hai nguồn cùng có số để kiểm chứng lẫn nhau.
+14/09 SỬA MỘT LỖI CỘNG ĐÔI trong bước gộp độ trễ: khoá dựng từ cột phẳng làm MỘT chuỗi bị cộng hai lần khi có hơn một lần kéo, và số lớn hơn trông y hệt số đúng. Chỉ lộ ra khi so với bản một-nguồn theo TỪNG KHOÁ.</t>
         </is>
       </c>
       <c r="K12" s="17" t="n"/>
@@ -1551,7 +1557,7 @@
       <c r="M12" s="17" t="n"/>
       <c r="N12" s="19" t="n"/>
       <c r="O12" s="19" t="n"/>
-      <c r="P12" s="17" t="n"/>
+      <c r="P12" s="53" t="n"/>
       <c r="Q12" s="17" t="n"/>
       <c r="R12" s="17" t="n"/>
       <c r="S12" s="17" t="n"/>
@@ -1614,14 +1620,15 @@
       </c>
       <c r="J13" s="55" t="inlineStr">
         <is>
-          <t>Khung 2 instance LiteLLM + nginx load balancer đã có trong docker-compose.yml từ 27/08, và 31/08 đã chạy lưu lượng THẬT qua khung này. Chưa có máy server thứ hai: cả 2 instance đang trên cùng một máy, nên chưa chứng minh được gì về chịu tải nhiều máy, cũng chưa thử thêm/bớt instance khi hệ thống đang chạy.</t>
+          <t>Khung 2 instance LiteLLM + nginx load balancer đã có trong docker-compose.yml từ 27/08, và 31/08 đã chạy lưu lượng THẬT qua khung này. Chưa có máy server thứ hai: cả 2 instance đang trên cùng một máy, nên chưa chứng minh được gì về chịu tải nhiều máy, cũng chưa thử thêm/bớt instance khi hệ thống đang chạy.
+07/09 ĐO SỨC CHỊU TẢI THẬT, trên sân riêng bốn lớp cách ly (mock trong cấu hình tuyến · database litellm_bench riêng · KHÔNG khai Redis · cổng 4003 không qua gateway-lb), cộng một bẫy cố ý: khoá Google của bench đặt sai để nếu mock không ăn thì nó hỏng ồn ào chứ không âm thầm tiêu tiền. CÁCH LY ĐƯỢC CHỨNG MINH, không phải tuyên bố: qua 51.223 lượt bench, SpendLogs thật 50→50, fact_call 8.672→8.672, fact_usage_daily 1.990→1.990. TRẦN ~150-170 req/s BẤT KỂ ĐỒNG THỜI: tăng số người dùng đồng thời gấp 2.000 lần (5 → 10.000) chỉ đổi được 28% thông lượng, phần tải thêm biến thành thời gian xếp hàng. HỆ KHÔNG GÃY — NÓ HOÁ THÀNH HÀNG ĐỢI: 0 kết nối bị từ chối; vài lỗi ở mức 5.000-8.000 đều là client không mở nổi kết nối chứ không phải server từ chối. Hệ quả phải ghi lại: QUÁ TẢI KHÔNG BÁO BẰNG LỖI, nó báo bằng người dùng ngồi đợi 38 giây — không sinh dòng cảnh báo nào. NÚT THẮT LÀ CPU CỦA LITELLM, KHÔNG PHẢI DATABASE: đo lúc đang tải, litellm-bench 105% (ghim chặt MỘT lõi trong 16 lõi container thấy được), postgres 0,4%. num_workers không được khai ở đâu cả, tức đang dùng 1/16 lõi — việc rẻ nhất chưa ai làm; 'tăng worker sẽ tăng thông lượng' vẫn là SUY LUẬN, chưa đo. Không làm OOM được bằng số kết nối: 120/120 mẫu 'running', OOMKilled=false; siết trần xuống 700 MB thì nó chạy bằng 264 MB. VẪN CHƯA CÓ MÁY SERVER THỨ HAI — toàn bộ phép đo trên MÁY DEV, hai instance cùng một máy, nên chưa chứng minh được gì về chịu tải nhiều máy và chưa thử thêm/bớt instance khi hệ thống đang chạy.</t>
         </is>
       </c>
       <c r="K13" s="17" t="n"/>
       <c r="L13" s="17" t="n"/>
       <c r="M13" s="17" t="n"/>
       <c r="N13" s="56" t="n"/>
-      <c r="O13" s="17" t="n"/>
+      <c r="O13" s="56" t="n"/>
       <c r="P13" s="17" t="n"/>
       <c r="Q13" s="17" t="n"/>
       <c r="R13" s="17" t="n"/>
@@ -1671,13 +1678,17 @@
 (dự kiến)</t>
         </is>
       </c>
-      <c r="J14" s="16" t="n"/>
+      <c r="J14" s="16" t="inlineStr">
+        <is>
+          <t>10/09 ĐO NHÁNH 429 bằng cách ép trần rpm: 1 trên tuyến CRM. GATEWAY KHÔNG CHE 429, NHƯNG HOÃN NÓ 123,7 GIÂY: num_retries: 3 khiến Gateway tự thử lại ba lần trước khi chịu trả lỗi cho người gọi. Đo từ phía NGƯỜI GỌI trên ba lượt liên tiếp: 124 · 123,8 · 123,6 giây — con số trong log (~60 s) chỉ là một phần cửa sổ, lấy nó là lấy nhầm. rpm: 1 KHÔNG phải 'một lượt mỗi phút' mà là 'không lượt nào': bộ đếm đọc được current_rpm 1.0 ở cả BẢY phút liên tiếp, không một lần về 0 — nên phép đo này là cảnh TUYẾN CHẾT HẲN, không phải cảnh chạm trần thoáng qua, và kết luận không được suy rộng ra cảnh sau. Trần chi phí chốt trước khi đo: tổng 32 lượt gọi, $0,216. Phát hiện ngoài kế hoạch, đắt hơn câu hỏi ban đầu: token suy nghĩ ăn 96% ngân sách đầu ra. CHƯA LÀM: cấu hình rpm/tpm thật cho từng project trên Router, cơ chế phân bổ theo hạn mức còn lại, và hàng đợi có độ trễ tăng dần.</t>
+        </is>
+      </c>
       <c r="K14" s="17" t="n"/>
       <c r="L14" s="17" t="n"/>
       <c r="M14" s="17" t="n"/>
       <c r="N14" s="17" t="n"/>
       <c r="O14" s="17" t="n"/>
-      <c r="P14" s="17" t="n"/>
+      <c r="P14" s="56" t="n"/>
       <c r="Q14" s="17" t="n"/>
       <c r="R14" s="17" t="n"/>
       <c r="S14" s="17" t="n"/>
@@ -1726,13 +1737,17 @@
 (dự kiến)</t>
         </is>
       </c>
-      <c r="J15" s="16" t="n"/>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>08/09 REDIS TỰ ĐỔI VAI: giết master thật thì replica thăng cấp sau 6 giây, 10/10 lượt 200 ngay sau đó (p50 0,99 s); chiều ngược 7 giây. Hai chiều đều chạy, không phải ăn may. 11-12/09 DIỄN TẬP MẤT GATEWAY trên 4 agent theo cùng một ma trận sáu bước: chạy nền qua LB → dừng MỘT Proxy để kiểm LB loại instance hỏng → khôi phục → dừng TOÀN BỘ LB để kiểm chính sách ứng dụng → khôi phục → đối soát response ID, định danh, token và SpendLogs. KẾT QUẢ KHÁC NHAU THEO CHÍNH SÁCH, và cả hai đều đúng: CRM tự chuyển sang gọi THẲNG nhà cung cấp sau ba lần mất kết nối liên tiếp, chạy xong lô đang dở, gửi đúng hai thư mỗi sự cố, KHÔNG mất dòng và KHÔNG đếm đôi; TLA-HĐ và Ralli thì FAIL-CLOSED có chủ ý — OCR không rơi sang Google hay Tesseract khi mất LB. gateway-lb được xác định là ĐIỂM HỎNG ĐƠN. CHƯA ĐẠT nên dòng này chưa tô xong: ba sentinel cùng một máy, hai instance LiteLLM cùng một máy, chưa có máy server thứ hai — mất máy là mất tất cả. Danh sách model dự phòng tự chuyển tuyến khi provider trả 5xx cũng chưa dựng.</t>
+        </is>
+      </c>
       <c r="K15" s="17" t="n"/>
       <c r="L15" s="17" t="n"/>
       <c r="M15" s="17" t="n"/>
       <c r="N15" s="17" t="n"/>
       <c r="O15" s="17" t="n"/>
-      <c r="P15" s="17" t="n"/>
+      <c r="P15" s="56" t="n"/>
       <c r="Q15" s="17" t="n"/>
       <c r="R15" s="17" t="n"/>
       <c r="S15" s="17" t="n"/>
@@ -1792,7 +1807,8 @@
       </c>
       <c r="J16" s="55" t="inlineStr">
         <is>
-          <t>Đang làm. 24/08 gỡ hết lọc cứng source='app' ở 10 chỗ đầu đọc. Chuyển schema sang v2 ĐÃ XONG (45/45 việc). 31/08 nguồn thứ tư vào database thật: fact_usage_daily có đủ 4 nguồn, gateway 1 ngày / 45.187 token; ba bộ số cũ KHÔNG đổi một token nào (đối soát 24 khoá mốc). 03/09 định nghĩa lại vế 2 cho đúng bản chất: đây là phép kiểm nội bộ, không phải báo cáo giao nộp. Đo: 0 ngày có đủ cả bốn nguồn — ngày duy nhất có Gateway (31/08) thì billing và monitoring đã dừng ở 29/08, app ở 30/08. Nên vế này KHÔNG chặn được bằng công sức. Ràng buộc "chạy song song tối thiểu 2 tuần trên agent production" GỠ KHỎI ĐƯỜNG GĂNG của STT 6 — nó vẫn là sản phẩm của STT 7 dòng 19, chỉ không còn chặn STT 6. Phép kiểm đối chiếu nay chạy được ngay: audit_db.py có 68 phép, trong đó nhóm F đối chiếu tổng theo giờ với tổng theo ngày CHO TỪNG NGUỒN, nhóm G đối chiếu chiều tài khoản với usage_resolved trên cả token lẫn calls, và ba phép chéo kiểm với /api/health qua một đường tính hoàn toàn khác. 04/09 đóng nốt đường NẠP: refresh_gateway.py trước đây chỉ làm mới 2 bảng trong số 4 bảng mà Gateway chạm tới, nên phân vị và bảng theo giờ giữ số cũ trong im lặng sau mỗi lần nạp. Nay 4 bước, và bản tóm tắt in đủ 4 bảng thay vì 2 (commit 131d3b5).</t>
+          <t>Đang làm. 24/08 gỡ hết lọc cứng source='app' ở 10 chỗ đầu đọc. Chuyển schema sang v2 ĐÃ XONG (45/45 việc). 31/08 nguồn thứ tư vào database thật: fact_usage_daily có đủ 4 nguồn, gateway 1 ngày / 45.187 token; ba bộ số cũ KHÔNG đổi một token nào (đối soát 24 khoá mốc). 03/09 định nghĩa lại vế 2 cho đúng bản chất: đây là phép kiểm nội bộ, không phải báo cáo giao nộp. Đo: 0 ngày có đủ cả bốn nguồn — ngày duy nhất có Gateway (31/08) thì billing và monitoring đã dừng ở 29/08, app ở 30/08. Nên vế này KHÔNG chặn được bằng công sức. Ràng buộc "chạy song song tối thiểu 2 tuần trên agent production" GỠ KHỎI ĐƯỜNG GĂNG của STT 6 — nó vẫn là sản phẩm của STT 7 dòng 19, chỉ không còn chặn STT 6. Phép kiểm đối chiếu nay chạy được ngay: audit_db.py có 68 phép, trong đó nhóm F đối chiếu tổng theo giờ với tổng theo ngày CHO TỪNG NGUỒN, nhóm G đối chiếu chiều tài khoản với usage_resolved trên cả token lẫn calls, và ba phép chéo kiểm với /api/health qua một đường tính hoàn toàn khác. 04/09 đóng nốt đường NẠP: refresh_gateway.py trước đây chỉ làm mới 2 bảng trong số 4 bảng mà Gateway chạm tới, nên phân vị và bảng theo giờ giữ số cũ trong im lặng sau mỗi lần nạp. Nay 4 bước, và bản tóm tắt in đủ 4 bảng thay vì 2 (commit 131d3b5).
+09/09 SỔ GATEWAY TỰ VỀ DASHBOARD, không cần ai chạy lệnh (nhịp tim làm mới, migration 012). 12/09 giãn nhịp lên 300 giây sau khi ĐO được 94% chu kỳ không dựng lại gì — phần lớn công việc trước đó là chạy không. 14/09 SỬA LUẬT GỘP, hai chỗ: lần kéo sau không còn làm TEO lần kéo trước (luật cũ 'bản mới thắng' gặp một lần kéo cụt ở mép cửa sổ là mất số), và dựng lại database không còn cần DROP SCHEMA. 14/09 BỎ HẲN database cũ token_ledger sau khi chứng minh v2 chứa đủ — nay chỉ còn một database.</t>
         </is>
       </c>
       <c r="K16" s="17" t="n"/>
@@ -1800,7 +1816,7 @@
       <c r="M16" s="56" t="n"/>
       <c r="N16" s="56" t="n"/>
       <c r="O16" s="17" t="n"/>
-      <c r="P16" s="17" t="n"/>
+      <c r="P16" s="56" t="n"/>
       <c r="Q16" s="17" t="n"/>
       <c r="R16" s="17" t="n"/>
       <c r="S16" s="17" t="n"/>
@@ -1850,7 +1866,8 @@
       </c>
       <c r="J17" s="16" t="inlineStr">
         <is>
-          <t>XONG 03/09/2026, sớm 34 ngày so với mốc. VẾ 1 — truy vấn và endpoint mới: GET /api/usage-hourly (bắt buộc có khoảng thời gian, khác 9 endpoint kia); /api/usage-by-account đọc view mới usage_by_account_resolved, phủ 8/8 agent thay vì 2/8 (1.453 dòng / 60 tài khoản); /api/performance đọc latency_resolved nên phân vị Gateway lên được dashboard — p95 ngày 31/08 = 1,822 s tính CHÍNH XÁC từ duration_ms thô thay vì nội suy trong ô histogram rộng trung bình 31,3 giây. VẾ 2 — kỷ luật chỉ-đọc: phát hiện và bịt một lỗ hổng chưa ai biết. rebuild_db.py bước 1 gọi DROP SCHEMA, xoá sạch GRANT của vai api_readonly, và CẢ HAI bộ kiểm đều báo lành trong lúc API mù — đo 02/09: container api chạy 38 phút trên database nó không đọc nổi. Nay rebuild_db.py có bước 10 kiểm quyền và DỪNG nếu thiếu; check_api.py hỏi MÁY CHỦ qua HTTP thay vì hỏi kết nối của chính nó. Tái tạo được lỗi: sau rebuild_db.py, api_readonly đọc 0/26 bảng+view, phép mới HỎNG còn phép cũ vẫn báo ĐẠT. Nghiệm thu: audit 68/64/4/0, check_api 27/27.</t>
+          <t>XONG 03/09/2026, sớm 34 ngày so với mốc. VẾ 1 — truy vấn và endpoint mới: GET /api/usage-hourly (bắt buộc có khoảng thời gian, khác 9 endpoint kia); /api/usage-by-account đọc view mới usage_by_account_resolved, phủ 8/8 agent thay vì 2/8 (1.453 dòng / 60 tài khoản); /api/performance đọc latency_resolved nên phân vị Gateway lên được dashboard — p95 ngày 31/08 = 1,822 s tính CHÍNH XÁC từ duration_ms thô thay vì nội suy trong ô histogram rộng trung bình 31,3 giây. VẾ 2 — kỷ luật chỉ-đọc: phát hiện và bịt một lỗ hổng chưa ai biết. rebuild_db.py bước 1 gọi DROP SCHEMA, xoá sạch GRANT của vai api_readonly, và CẢ HAI bộ kiểm đều báo lành trong lúc API mù — đo 02/09: container api chạy 38 phút trên database nó không đọc nổi. Nay rebuild_db.py có bước 10 kiểm quyền và DỪNG nếu thiếu; check_api.py hỏi MÁY CHỦ qua HTTP thay vì hỏi kết nối của chính nó. Tái tạo được lỗi: sau rebuild_db.py, api_readonly đọc 0/26 bảng+view, phép mới HỎNG còn phép cũ vẫn báo ĐẠT. Nghiệm thu: audit 68/64/4/0, check_api 27/27.
+14/09 ĐÓNG NỐT LỖ HỔNG GRANT ghi ở trên, theo đường gốc: bước dựng lại database không còn gọi DROP SCHEMA, nên không còn cửa nào xoá GRANT của vai api_readonly. Trước đó bước 10 chỉ BẮT được lỗi sau khi nó đã xảy ra; nay cửa đó đóng lại.</t>
         </is>
       </c>
       <c r="K17" s="17" t="n"/>
@@ -1858,7 +1875,7 @@
       <c r="M17" s="17" t="n"/>
       <c r="N17" s="19" t="n"/>
       <c r="O17" s="19" t="n"/>
-      <c r="P17" s="17" t="n"/>
+      <c r="P17" s="53" t="n"/>
       <c r="Q17" s="17" t="n"/>
       <c r="R17" s="17" t="n"/>
       <c r="S17" s="17" t="n"/>
@@ -1907,7 +1924,8 @@
       </c>
       <c r="J18" s="16" t="inlineStr">
         <is>
-          <t>Đang làm. 30/08/2026 commit 2f5b34d nối lại phần hiển thị user / phòng ban với database (+357 dòng web/js/app.js, +84 dòng web/js/api.js, thêm bộ kiểm filter-select-refresh). Dữ liệu nền đã đủ: cả 8/8 agent đều có số trong fact_usage_daily. 03/09 — 2/3 biểu đồ XONG. View usage_by_account_resolved phủ 8/8 agent (1.453 dòng / 60 tài khoản / token 915.969.971 và calls 122.504, cả hai khớp usage_resolved). ① Tỷ lệ áp dụng: XONG, 8/8 agent — sáu agent dịch vụ mẫu số 1 là ĐÚNG theo quy ước account chốt 20/08; câu chữ "theo phòng ban" đã sửa thành "theo agent". ② Người dùng hoạt động theo ngày: XONG, từ 2/8 lên 8/8 agent — đường cong sẽ nhảy lên vì dữ liệu mới, không phải lỗi; đây là đếm TÀI KHOẢN chứ không phải người ngoài đời. ③ Chi phí theo phòng ban: CHƯA — donut vẫn khoá theo primaryUnit(), tức đơn vị GỐC của agent, nên 130 đơn vị chỉ ra 8 lát: sáu lát là tên agent đổi nhãn, hai lát là gốc cây (cả công ty). Không lát nào là một phòng ban. Tiền thì CÓ (từ /api/usage), cái sai là chiều phòng ban. Muốn đúng thì cần cost_usd xuống tới mức tài khoản, mà tiền chỉ tồn tại ở mức (ngày, agent, model) — chia đều cho các tài khoản là bịa. Việc này chưa nằm trong change nào.</t>
+          <t>Đang làm. 30/08/2026 commit 2f5b34d nối lại phần hiển thị user / phòng ban với database (+357 dòng web/js/app.js, +84 dòng web/js/api.js, thêm bộ kiểm filter-select-refresh). Dữ liệu nền đã đủ: cả 8/8 agent đều có số trong fact_usage_daily. 03/09 — 2/3 biểu đồ XONG. View usage_by_account_resolved phủ 8/8 agent (1.453 dòng / 60 tài khoản / token 915.969.971 và calls 122.504, cả hai khớp usage_resolved). ① Tỷ lệ áp dụng: XONG, 8/8 agent — sáu agent dịch vụ mẫu số 1 là ĐÚNG theo quy ước account chốt 20/08; câu chữ "theo phòng ban" đã sửa thành "theo agent". ② Người dùng hoạt động theo ngày: XONG, từ 2/8 lên 8/8 agent — đường cong sẽ nhảy lên vì dữ liệu mới, không phải lỗi; đây là đếm TÀI KHOẢN chứ không phải người ngoài đời. ③ Chi phí theo phòng ban: CHƯA — donut vẫn khoá theo primaryUnit(), tức đơn vị GỐC của agent, nên 130 đơn vị chỉ ra 8 lát: sáu lát là tên agent đổi nhãn, hai lát là gốc cây (cả công ty). Không lát nào là một phòng ban. Tiền thì CÓ (từ /api/usage), cái sai là chiều phòng ban. Muốn đúng thì cần cost_usd xuống tới mức tài khoản, mà tiền chỉ tồn tại ở mức (ngày, agent, model) — chia đều cho các tài khoản là bịa. Việc này chưa nằm trong change nào.
+10-11/09 RÀ LẠI GIAO DIỆN theo góp ý 25/07. Tám thẻ KPI gom về MỘT bộ dựng thay vì tám nhánh riêng, và phân biệt được hai cảnh trước đây hiện như nhau: 'không có kỳ so sánh' khác 'kỳ so sánh đo được bằng 0'. Biểu đồ ngân sách BỎ HẲN agent mà bộ lọc đã loại, thay vì vẽ chúng ở mức 0 — vẽ ở 0 là nói agent đó không tiêu gì. Bộ lọc người dùng nay NÓI RÕ nó đang giấu gì thay vì lặng lẽ bỏ đi. Đánh dấu agent tiêu cao hơn 30% mức trung bình và nói tiền đó từ đâu ra. Vẽ tỷ lệ lỗi theo agent/nhóm lỗi. BỎ lời hứa phân vị mà tab Hiệu năng chưa bao giờ đo — gỡ một con số bịa khỏi giao diện. ③ CHI PHÍ THEO PHÒNG BAN VẪN CHƯA: 15/09 mới có KẾ HOẠCH và hai phương án phác thảo giao diện lọc phòng ban/đơn vị, chưa dựng. Nguyên nhân gốc KHÔNG đổi: tiền chỉ tồn tại ở mức (ngày, agent, model), chia đều xuống tài khoản là bịa.</t>
         </is>
       </c>
       <c r="K18" s="17" t="n"/>
@@ -1915,8 +1933,8 @@
       <c r="M18" s="17" t="n"/>
       <c r="N18" s="56" t="n"/>
       <c r="O18" s="17" t="n"/>
-      <c r="P18" s="17" t="n"/>
-      <c r="Q18" s="17" t="n"/>
+      <c r="P18" s="56" t="n"/>
+      <c r="Q18" s="56" t="n"/>
       <c r="R18" s="17" t="n"/>
       <c r="S18" s="17" t="n"/>
       <c r="T18" s="17" t="n"/>
@@ -1974,7 +1992,11 @@
 (dự kiến)</t>
         </is>
       </c>
-      <c r="J19" s="16" t="n"/>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu kỳ chạy song song. ĐIỀU KIỆN CHẶN, ghi lại để không ai tưởng đây là việc soạn báo cáo: kỳ này cần Gateway và ba nguồn cũ cùng có dữ liệu tối thiểu 2 tuần, mà tính đến 16/09 mới 1/8 agent chạy production qua Gateway. Ngưỡng chấp nhận sai lệch và quy trình xử lý khi vượt ngưỡng cũng CHƯA ban hành — và theo đúng kỷ luật ghi ở chính dòng này, chúng phải ban hành TRƯỚC kỳ đo, không phải sau khi đã nhìn thấy số.</t>
+        </is>
+      </c>
       <c r="K19" s="17" t="n"/>
       <c r="L19" s="17" t="n"/>
       <c r="M19" s="17" t="n"/>
@@ -2030,7 +2052,8 @@
       </c>
       <c r="J20" s="55" t="inlineStr">
         <is>
-          <t>Đang làm. 31/08 scripts/audit_db.py đã có phép kiểm cho nguồn gateway: lượt hỏng không lọt vào bảng tổng hợp, không dòng nào có duration_ms = 0, không có giá trị outcome lạ. Chạy 01/09: 39 phép kiểm, 35 đạt, 4 lưu ý (đều là thiếu dữ liệu đã biết), 0 hỏng. 03/09: audit_db.py thêm nhóm F (12 phép) — tổng giờ khớp tổng ngày theo từng nguồn, không có billing trong bảng giờ, mọi giờ cắt đúng đầu giờ, phân vị số thô không mang ô histogram và ngược lại phân vị nội suy phải giữ ô. Chạy đầy đủ: 54 phép / 50 đạt / 4 lưu ý / 0 hỏng. backend/check_api.py XONG: thêm 6 phép cho endpoint theo giờ, chạy 25/25 đạt. Trong lúc làm, phát hiện check_api.py mang một phép kiểm LỖI THỜI từ 31/08 — nó so tiền API với riêng fact_billing_daily trong khi migration 005 đã cố ý đổ tiền Gateway vào usage_resolved ($307,360850 + $0,021305 = $307,382155), nên nó báo HỎNG cho một hệ thống đang đúng; đã sửa CÔNG THỨC theo đúng phép của audit_db.py, không nới ngưỡng. 03/09 chiều — XONG cả hai vế, nhưng vế 2 XONG theo nghĩa PHÉP KIỂM ĐÃ CÓ VÀ NÓ NÓI THẲNG LÀ CHƯA KIỂM ĐƯỢC, không phải theo nghĩa đã đối chiếu xong. VẾ 1 — bốn phép mà mục này liệt kê: KHOÁ NGOẠI nay đọc từ pg_constraint thay vì một danh sách gõ tay; đo được danh sách cũ đã trôi mất 13/36 quan hệ, trong đó 6 do chính migration 008 tạo ra sáng cùng ngày — nó tụt trong im lặng vì nhãn vẫn báo "Foreign keys (23 relations)" ĐẠT, mà 23 là số quan hệ ĐƯỢC KHAI chứ không phải số CÓ THẬT. Thêm mốc số lượng (&gt;= 36) để bắt chiều ngược lại: xoá một khoá ngoại thì danh sách tự sinh vẫn xanh. NGÀY TƯƠNG LAI bỏ ngưỡng ghim '2026-12-31' (sang 2027 mọi dòng thật đều bị coi là tương lai), thay bằng CURRENT_DATE + 1, và soi 5 bảng thay vì 1 — kể cả fact_call, nơi Gateway ghi từng lượt. TÀI KHOẢN LẠ và SỐ KHỚP HOÁ ĐƠN đã có từ 31/08, nay bổ sung mẫu số quan sát. VẾ 2 — phép kiểm đối chiếu token cache ĐÃ VIẾT XONG (nhóm H của audit_db.py), so theo ngày × agent trên đúng những ngày CẢ HAI nguồn cùng có, ngưỡng 1% chốt TRƯỚC kỳ đo theo đúng kỷ luật STT 7 dòng 19. Chạy hôm nay ra CHƯA KIỂM ĐƯỢC: gateway 31/08→31/08 (1 ngày), hoá đơn 05/01→29/08 (214 ngày), SỐ NGÀY GIAO NHAU = 0; và vế Gateway rỗng sạch (cached_tokens 0/41). ĐIỀU KIỆN ĐỂ NÓ CHẠY: một ngày mà Gateway và hoá đơn Google cùng có dữ liệu — hoá đơn về trễ ~1 ngày nên chỉ cần Gateway chạy thêm vài ngày liên tục là đủ. SỬA MỘT HÌNH DẠNG LỖI, không chỉ thêm phép kiểm: mọi phép kiểm theo nguồn nay khai CẢ MẪU SỐ. Trước đây "0 dòng xấu" trên 0 dòng gateway báo ĐẠT — nó không phân biệt "Gateway ghi đúng" với "Gateway không ghi gì cả", và đó đúng là hình dạng đã để API mù 38 phút ngày 02/09. Nghiệm thu bằng cách tái tạo trên một tập rỗng THẬT (fact_perf_daily không có dòng gateway nào), không dựng database giả. NGHIỆM THU: audit_db.py 72 phép / 65 đạt / 7 lưu ý / 0 hỏng (mốc 68/64/4/0 — lưu ý tăng 4→7 là ĐÚNG, ba cái mới đều là chỗ trước nay báo đạt mà chưa quan sát gì, và bốn lưu ý cũ giữ nguyên); check_api.py 31/31 (mốc 27/27); chạy hai lần liên tiếp số không đổi; usage_resolved khớp 4/4 khoá — change này không đụng một dòng dữ liệu nào. ĐÍNH CHÍNH 04/09: con số nghiệm thu ghi ở trên là 72/65/7/0, đo TRƯỚC commit 131d3b5 của cùng ngày 03/09. Sau commit đó bộ kiểm có thêm một phép (các bảng dẫn xuất từ Gateway phải mới ngang fact_call), nên mốc đúng là 73 phép / 66 đạt / 7 lưu ý / 0 hỏng. check_api.py giữ nguyên 31/31. 05/09 THÊM HAI NHÓM PHÉP KIỂM. NHÓM I — đối chiếu fact_call với số của CHÍNH NHÀ CUNG CẤP (bảng mới fact_provider_daily, migration 011), trên CẢ BA TRỤC và ở MỨC NGÀY. Ba trục chứ không một, vì ngày 31/08 số lượt khớp tuyệt đối 41/41 trong khi token lệch 6.334 — kiểm mỗi trục số lượt là phép kiểm xanh và lỗi đi qua. Mức ngày chứ không mức giờ, vì nhà cung cấp gắn nhãn ô theo thời điểm KẾT THÚC còn sổ ta ghi theo thời điểm BẮT ĐẦU: đo được giờ 01 lệch +1 lượt và giờ 02 lệch −1, cộng lại bằng 0 — một request rơi hai ô, không phải hai lỗi. HAI CHIỀU LỆCH XỬ LÝ KHÁC NHAU: nhà cung cấp nhiều hơn ta là chiều KỲ VỌNG nên LƯU Ý kèm số tuyệt đối và tỷ lệ, MUST NOT báo hỏng (báo hỏng thì phép kiểm đỏ vĩnh viễn rồi bị bỏ qua); ta nhiều hơn nhà cung cấp là HỎNG, không ngưỡng, vì ta không thể tiêu thứ họ không phục vụ. CHƯA ĐẶT NGƯỠNG PHẦN TRĂM cho chiều thiếu hụt, và đó là CHỦ Ý: đã biết đáp án 12,21% rồi mới viết phép kiểm, nên đặt ngưỡng bây giờ là chọn số vừa khít với đáp án — trái kỷ luật "ban hành ngưỡng trước kỳ đo" đã chốt ở dòng 19. NGHIỆM THU CHIỀU HỎNG BẰNG CÁCH TÁI TẠO LỖI, không chỉ đọc code: hạ vế nhà cung cấp xuống dưới fact_call thì audit đỏ đúng cả ba trục và thoát mã 1; nạp lại từ đợt kéo thì về nguyên trạng từng byte và xanh lại. NHÓM J — kế toán từng dòng sổ nguồn, TỰ TÍNH LẠI bằng SQL của riêng nó thay vì tin lời bộ nạp. HỎNG khi một dòng lẽ ra nạp được mà vắng mặt, và cả chiều ngược lại: dòng có trong fact_call mà sổ nguồn không còn. Đo được 47 dòng nguồn = 41 nạp + 5 không có tag định danh (408 token) + 1 bản sao cú cache hit (352 token), 0 dòng không giải thích được. Bản sao cache hit là phát hiện ngoài kế hoạch: LiteLLM ghi thêm một dòng mang request_id gốc cộng hậu tố _cache_hit&lt;epoch&gt; và LẶP LẠI nguyên token; hôm nay nó rớt vì một lý do chẳng liên quan, nên load_gateway.py nay loại nó tường minh — nếu không, ngày nào khâu định danh được nới ra là đếm đôi 352 token mà không phép kiểm nào bắt được. HỆ QUẢ CHO VẾ 2 CỦA MỤC NÀY: phép kiểm cache nhóm H sẽ KHÔNG BAO GIỜ chạy được cho lưu lượng Gateway, vì khoá là free tier nên không lên hoá đơn — nó vẫn đúng cho lưu lượng agent trả tiền. NGHIỆM THU: audit_db.py 78 phép / 68 đạt / 10 lưu ý / 0 hỏng (mốc 73/66/7/0 — tăng đúng 5 phép: nhóm I 2, nhóm J 3); chạy hai lần liên tiếp số không đổi; usage_resolved khớp 4/4 khoá mốc.</t>
+          <t>Đang làm. 31/08 scripts/audit_db.py đã có phép kiểm cho nguồn gateway: lượt hỏng không lọt vào bảng tổng hợp, không dòng nào có duration_ms = 0, không có giá trị outcome lạ. Chạy 01/09: 39 phép kiểm, 35 đạt, 4 lưu ý (đều là thiếu dữ liệu đã biết), 0 hỏng. 03/09: audit_db.py thêm nhóm F (12 phép) — tổng giờ khớp tổng ngày theo từng nguồn, không có billing trong bảng giờ, mọi giờ cắt đúng đầu giờ, phân vị số thô không mang ô histogram và ngược lại phân vị nội suy phải giữ ô. Chạy đầy đủ: 54 phép / 50 đạt / 4 lưu ý / 0 hỏng. backend/check_api.py XONG: thêm 6 phép cho endpoint theo giờ, chạy 25/25 đạt. Trong lúc làm, phát hiện check_api.py mang một phép kiểm LỖI THỜI từ 31/08 — nó so tiền API với riêng fact_billing_daily trong khi migration 005 đã cố ý đổ tiền Gateway vào usage_resolved ($307,360850 + $0,021305 = $307,382155), nên nó báo HỎNG cho một hệ thống đang đúng; đã sửa CÔNG THỨC theo đúng phép của audit_db.py, không nới ngưỡng. 03/09 chiều — XONG cả hai vế, nhưng vế 2 XONG theo nghĩa PHÉP KIỂM ĐÃ CÓ VÀ NÓ NÓI THẲNG LÀ CHƯA KIỂM ĐƯỢC, không phải theo nghĩa đã đối chiếu xong. VẾ 1 — bốn phép mà mục này liệt kê: KHOÁ NGOẠI nay đọc từ pg_constraint thay vì một danh sách gõ tay; đo được danh sách cũ đã trôi mất 13/36 quan hệ, trong đó 6 do chính migration 008 tạo ra sáng cùng ngày — nó tụt trong im lặng vì nhãn vẫn báo "Foreign keys (23 relations)" ĐẠT, mà 23 là số quan hệ ĐƯỢC KHAI chứ không phải số CÓ THẬT. Thêm mốc số lượng (&gt;= 36) để bắt chiều ngược lại: xoá một khoá ngoại thì danh sách tự sinh vẫn xanh. NGÀY TƯƠNG LAI bỏ ngưỡng ghim '2026-12-31' (sang 2027 mọi dòng thật đều bị coi là tương lai), thay bằng CURRENT_DATE + 1, và soi 5 bảng thay vì 1 — kể cả fact_call, nơi Gateway ghi từng lượt. TÀI KHOẢN LẠ và SỐ KHỚP HOÁ ĐƠN đã có từ 31/08, nay bổ sung mẫu số quan sát. VẾ 2 — phép kiểm đối chiếu token cache ĐÃ VIẾT XONG (nhóm H của audit_db.py), so theo ngày × agent trên đúng những ngày CẢ HAI nguồn cùng có, ngưỡng 1% chốt TRƯỚC kỳ đo theo đúng kỷ luật STT 7 dòng 19. Chạy hôm nay ra CHƯA KIỂM ĐƯỢC: gateway 31/08→31/08 (1 ngày), hoá đơn 05/01→29/08 (214 ngày), SỐ NGÀY GIAO NHAU = 0; và vế Gateway rỗng sạch (cached_tokens 0/41). ĐIỀU KIỆN ĐỂ NÓ CHẠY: một ngày mà Gateway và hoá đơn Google cùng có dữ liệu — hoá đơn về trễ ~1 ngày nên chỉ cần Gateway chạy thêm vài ngày liên tục là đủ. SỬA MỘT HÌNH DẠNG LỖI, không chỉ thêm phép kiểm: mọi phép kiểm theo nguồn nay khai CẢ MẪU SỐ. Trước đây "0 dòng xấu" trên 0 dòng gateway báo ĐẠT — nó không phân biệt "Gateway ghi đúng" với "Gateway không ghi gì cả", và đó đúng là hình dạng đã để API mù 38 phút ngày 02/09. Nghiệm thu bằng cách tái tạo trên một tập rỗng THẬT (fact_perf_daily không có dòng gateway nào), không dựng database giả. NGHIỆM THU: audit_db.py 72 phép / 65 đạt / 7 lưu ý / 0 hỏng (mốc 68/64/4/0 — lưu ý tăng 4→7 là ĐÚNG, ba cái mới đều là chỗ trước nay báo đạt mà chưa quan sát gì, và bốn lưu ý cũ giữ nguyên); check_api.py 31/31 (mốc 27/27); chạy hai lần liên tiếp số không đổi; usage_resolved khớp 4/4 khoá — change này không đụng một dòng dữ liệu nào. ĐÍNH CHÍNH 04/09: con số nghiệm thu ghi ở trên là 72/65/7/0, đo TRƯỚC commit 131d3b5 của cùng ngày 03/09. Sau commit đó bộ kiểm có thêm một phép (các bảng dẫn xuất từ Gateway phải mới ngang fact_call), nên mốc đúng là 73 phép / 66 đạt / 7 lưu ý / 0 hỏng. check_api.py giữ nguyên 31/31. 05/09 THÊM HAI NHÓM PHÉP KIỂM. NHÓM I — đối chiếu fact_call với số của CHÍNH NHÀ CUNG CẤP (bảng mới fact_provider_daily, migration 011), trên CẢ BA TRỤC và ở MỨC NGÀY. Ba trục chứ không một, vì ngày 31/08 số lượt khớp tuyệt đối 41/41 trong khi token lệch 6.334 — kiểm mỗi trục số lượt là phép kiểm xanh và lỗi đi qua. Mức ngày chứ không mức giờ, vì nhà cung cấp gắn nhãn ô theo thời điểm KẾT THÚC còn sổ ta ghi theo thời điểm BẮT ĐẦU: đo được giờ 01 lệch +1 lượt và giờ 02 lệch −1, cộng lại bằng 0 — một request rơi hai ô, không phải hai lỗi. HAI CHIỀU LỆCH XỬ LÝ KHÁC NHAU: nhà cung cấp nhiều hơn ta là chiều KỲ VỌNG nên LƯU Ý kèm số tuyệt đối và tỷ lệ, MUST NOT báo hỏng (báo hỏng thì phép kiểm đỏ vĩnh viễn rồi bị bỏ qua); ta nhiều hơn nhà cung cấp là HỎNG, không ngưỡng, vì ta không thể tiêu thứ họ không phục vụ. CHƯA ĐẶT NGƯỠNG PHẦN TRĂM cho chiều thiếu hụt, và đó là CHỦ Ý: đã biết đáp án 12,21% rồi mới viết phép kiểm, nên đặt ngưỡng bây giờ là chọn số vừa khít với đáp án — trái kỷ luật "ban hành ngưỡng trước kỳ đo" đã chốt ở dòng 19. NGHIỆM THU CHIỀU HỎNG BẰNG CÁCH TÁI TẠO LỖI, không chỉ đọc code: hạ vế nhà cung cấp xuống dưới fact_call thì audit đỏ đúng cả ba trục và thoát mã 1; nạp lại từ đợt kéo thì về nguyên trạng từng byte và xanh lại. NHÓM J — kế toán từng dòng sổ nguồn, TỰ TÍNH LẠI bằng SQL của riêng nó thay vì tin lời bộ nạp. HỎNG khi một dòng lẽ ra nạp được mà vắng mặt, và cả chiều ngược lại: dòng có trong fact_call mà sổ nguồn không còn. Đo được 47 dòng nguồn = 41 nạp + 5 không có tag định danh (408 token) + 1 bản sao cú cache hit (352 token), 0 dòng không giải thích được. Bản sao cache hit là phát hiện ngoài kế hoạch: LiteLLM ghi thêm một dòng mang request_id gốc cộng hậu tố _cache_hit&lt;epoch&gt; và LẶP LẠI nguyên token; hôm nay nó rớt vì một lý do chẳng liên quan, nên load_gateway.py nay loại nó tường minh — nếu không, ngày nào khâu định danh được nới ra là đếm đôi 352 token mà không phép kiểm nào bắt được. HỆ QUẢ CHO VẾ 2 CỦA MỤC NÀY: phép kiểm cache nhóm H sẽ KHÔNG BAO GIỜ chạy được cho lưu lượng Gateway, vì khoá là free tier nên không lên hoá đơn — nó vẫn đúng cho lưu lượng agent trả tiền. NGHIỆM THU: audit_db.py 78 phép / 68 đạt / 10 lưu ý / 0 hỏng (mốc 73/66/7/0 — tăng đúng 5 phép: nhóm I 2, nhóm J 3); chạy hai lần liên tiếp số không đổi; usage_resolved khớp 4/4 khoá mốc.
+13/09 BỘ KIỂM NAY CHẠY MỖI LẦN PUSH, không còn phụ thuộc ai nhớ chạy tay. Bốn nhóm chạy song song: Canh cấu hình · Phép kiểm JavaScript (chốt 53) · Phép kiểm Python (chốt 58) · Gateway image. Bộ kiểm BÁO SỐ phép kiểm và đỏ nếu lệch mốc, nên một mẫu tên tệp nở hụt không còn đi qua trong im lặng. NGHIỆM THU BẰNG CÁCH LÀM ĐỎ CÓ CHỦ Ý: hỏng lần lượt cả ba nhóm, xác nhận CI đỏ, rồi hoàn tác. Phát hiện trong lúc làm: một dấu ống nuốt mất mã thoát khiến job LUÔN xanh — đúng hình dạng lỗi 'phép kiểm không thể đỏ' đã gặp ngày 02/09. Ba cổng cấu hình: không tệp theo git nào ghim IP của một môi trường, địa chỉ bind đọc từ biến, và image Gateway phải đến từ registry chứ không build tại chỗ. Lần chạy 16/09 trên main: 4/4 nhóm xanh, 17 giây.</t>
         </is>
       </c>
       <c r="K20" s="17" t="n"/>
@@ -2038,8 +2061,8 @@
       <c r="M20" s="17" t="n"/>
       <c r="N20" s="56" t="n"/>
       <c r="O20" s="56" t="n"/>
-      <c r="P20" s="17" t="n"/>
-      <c r="Q20" s="17" t="n"/>
+      <c r="P20" s="56" t="n"/>
+      <c r="Q20" s="56" t="n"/>
       <c r="R20" s="17" t="n"/>
       <c r="S20" s="17" t="n"/>
       <c r="T20" s="17" t="n"/>
@@ -2086,13 +2109,17 @@
 (dự kiến)</t>
         </is>
       </c>
-      <c r="J21" s="16" t="n"/>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>07/09 BÁO CÁO THÔNG LƯỢNG đã có — xem dòng 13: trần ~150-170 req/s, nút thắt là CPU LiteLLM một lõi, quá tải biểu hiện bằng chờ 38 giây chứ không bằng lỗi. BA KỊCH BẢN SỰ CỐ mục này liệt kê nay ĐỀU ĐÃ ĐO: ① tắt 1 instance — dừng một Proxy, LB loại nó khỏi vòng chia lượt, khôi phục thì gọi lại bình thường (đo trên 4 agent, 11-12/09); ② tắt Redis — Gateway vẫn phục vụ 9/10 lượt, p50 0,87 s, giá phải trả là MỘT lần 5,12 s lúc client phát hiện mất kết nối, bật lại không phải làm gì, 0 lỗi tồn dư (07/09); ③ provider trả 429 — Gateway không che nhưng hoãn 123,7 giây, xem dòng 14 (10/09). CHƯA ĐỦ ĐỂ TÔ XONG, hai lý do: (a) phép đo thông lượng chạy trên MOCK và trên máy dev, nên chưa nói được ĐỘ TRỄ TĂNG THÊM DO GATEWAY trên tuyến thật — đã quan sát một lượt qua Gateway mất 81 giây trong khi gọi thẳng cùng lúc chỉ 1,4 giây, KHÔNG TÁI HIỆN ĐƯỢC và chưa rõ nguyên nhân; (b) kịch bản ③ chưa có kết quả mong đợi ghi TRƯỚC, ngưỡng vẫn chưa ban hành, nên nó là phép đo chứ chưa phải phép nghiệm thu.</t>
+        </is>
+      </c>
       <c r="K21" s="17" t="n"/>
       <c r="L21" s="17" t="n"/>
       <c r="M21" s="17" t="n"/>
       <c r="N21" s="17" t="n"/>
-      <c r="O21" s="17" t="n"/>
-      <c r="P21" s="17" t="n"/>
+      <c r="O21" s="56" t="n"/>
+      <c r="P21" s="56" t="n"/>
       <c r="Q21" s="17" t="n"/>
       <c r="R21" s="17" t="n"/>
       <c r="S21" s="17" t="n"/>
@@ -2150,9 +2177,10 @@
 (dự kiến)</t>
         </is>
       </c>
-      <c r="J22" s="57" t="inlineStr">
-        <is>
-          <t>Đang làm. 31/08/2026 chuyển agent ĐẦU TIÊN (dms-feedback, chọn vì ít lưu lượng nhất theo đúng tiêu chí dòng này) qua Gateway thật: Virtual Key riêng mang tag "dms-feedback", đo bằng ba dấu vết độc lập trên 10 lượt gọi — 7/8 thành công, 1/8 trượt đúng vào tuyến mồi (kỳ vọng, không phải lỗi). Số của agent này đã vào fact_usage_daily với source='gateway' và qua được audit_db.py. 1/8 agent — 7 agent còn lại (Trợ lý ảo Ralli, Trợ Lý Ảo Hợp Đồng, Phân Loại Dữ Liệu CRM, Chatbot Contact Center, Sale Agent, Multi modal AI Invoice, Tools Quizzer) vẫn gọi thẳng nhà cung cấp, chưa có Virtual Key thật — chờ điều kiện ① (8 khoá API của 8 project) theo docs/reference/ke-hoach-nen-thang-9-2026.md. (trên một agent) — phép đo và phép kiểm ở trên mới xác nhận đúng cho 1/8 agent; dòng này chỉ tính XONG (tô xanh) khi cả 8 agent cùng chạy qua Gateway, không phải khi suy rộng từ kết quả của một agent duy nhất.</t>
+      <c r="J22" s="16" t="inlineStr">
+        <is>
+          <t>Đang làm. 31/08/2026 chuyển agent ĐẦU TIÊN (dms-feedback, chọn vì ít lưu lượng nhất theo đúng tiêu chí dòng này) qua Gateway thật: Virtual Key riêng mang tag "dms-feedback", đo bằng ba dấu vết độc lập trên 10 lượt gọi — 7/8 thành công, 1/8 trượt đúng vào tuyến mồi (kỳ vọng, không phải lỗi). Số của agent này đã vào fact_usage_daily với source='gateway' và qua được audit_db.py. 1/8 agent — 7 agent còn lại (Trợ lý ảo Ralli, Trợ Lý Ảo Hợp Đồng, Phân Loại Dữ Liệu CRM, Chatbot Contact Center, Sale Agent, Multi modal AI Invoice, Tools Quizzer) vẫn gọi thẳng nhà cung cấp, chưa có Virtual Key thật — chờ điều kiện ① (8 khoá API của 8 project) theo docs/reference/ke-hoach-nen-thang-9-2026.md. (trên một agent) — phép đo và phép kiểm ở trên mới xác nhận đúng cho 1/8 agent; dòng này chỉ tính XONG (tô xanh) khi cả 8 agent cùng chạy qua Gateway, không phải khi suy rộng từ kết quả của một agent duy nhất.
+09-14/09 CRM là agent THỨ HAI được nối vào Gateway, nhưng phải đọc đúng mức: mới ở tầng HARNESS, chưa phải đường chạy theo lịch. Phần đo được là thật: gọi qua Vertex express ra 200, prompt thật 10.181 ký tự trong 2,75 giây, JSON phân tích được bằng CHÍNH hàm của CRM, sổ ghi model gemini/gemini-2.5-flash · 4.009 token · end_user svc.crm-feedback · tag crm-feedback. Đường chạy theo lịch thật CHƯA chạy vì đã cố ý chặn SharePoint/Excel/email trong lúc thử. Nên tính đến 16/09 vẫn là 1/8 agent chạy PRODUCTION (DMS, từ 31/08). Báo cáo hợp nhất 4 agent (TLA-HĐ · Ralli · DMS · CRM) ghi thẳng: KHÔNG agent nào được chứng nhận production-ready từ báo cáo đó — chưa nghiệm thu trên máy chủ thật, chưa TLS/allowlist, chưa chạy trọn tuyến SpendLogs → token_ledger_v2 → dashboard. Các phép đo khác tầng KHÔNG được cộng thành một con số chung.</t>
         </is>
       </c>
       <c r="K22" s="17" t="n"/>
@@ -2160,7 +2188,7 @@
       <c r="M22" s="17" t="n"/>
       <c r="N22" s="58" t="n"/>
       <c r="O22" s="58" t="n"/>
-      <c r="P22" s="17" t="n"/>
+      <c r="P22" s="56" t="n"/>
       <c r="Q22" s="17" t="n"/>
       <c r="R22" s="17" t="n"/>
       <c r="S22" s="17" t="n"/>

</xml_diff>